<commit_message>
Update poverty, education, ghg intensity
</commit_message>
<xml_diff>
--- a/intermediate/dashboard_output_SDG4.xlsx
+++ b/intermediate/dashboard_output_SDG4.xlsx
@@ -499,10 +499,10 @@
         </is>
       </c>
       <c r="H3">
-        <v>-1.617399042950514</v>
+        <v>-1.406539538892481</v>
       </c>
       <c r="I3">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J3">
         <v>4.4</v>
@@ -524,7 +524,7 @@
         <v>2015</v>
       </c>
       <c r="O3">
-        <v>7.541318681318685</v>
+        <v>7.672435897435901</v>
       </c>
     </row>
     <row r="4">
@@ -553,10 +553,10 @@
         </is>
       </c>
       <c r="H4">
-        <v>-1.498015873015875</v>
+        <v>-1.307539682539684</v>
       </c>
       <c r="I4">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J4">
         <v>8.6</v>
@@ -578,7 +578,7 @@
         <v>2015</v>
       </c>
       <c r="O4">
-        <v>10.13714285714286</v>
+        <v>10.18333333333334</v>
       </c>
     </row>
     <row r="5">
@@ -607,10 +607,10 @@
         </is>
       </c>
       <c r="H5">
-        <v>-3.125</v>
+        <v>-2.499999999999999</v>
       </c>
       <c r="I5">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J5">
         <v>12</v>
@@ -632,7 +632,7 @@
         <v>2015</v>
       </c>
       <c r="O5">
-        <v>12.38</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="6">
@@ -661,10 +661,10 @@
         </is>
       </c>
       <c r="H6">
-        <v>4.166666666666664</v>
+        <v>3.499999999999997</v>
       </c>
       <c r="I6">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J6">
         <v>12.1</v>
@@ -686,7 +686,7 @@
         <v>2015</v>
       </c>
       <c r="O6">
-        <v>11.54</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="7">
@@ -799,10 +799,10 @@
         </is>
       </c>
       <c r="H9">
-        <v>1.770833333333332</v>
+        <v>1.583333333333331</v>
       </c>
       <c r="I9">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J9">
         <v>11.5</v>
@@ -824,7 +824,7 @@
         <v>2015</v>
       </c>
       <c r="O9">
-        <v>11.315</v>
+        <v>11.325</v>
       </c>
     </row>
     <row r="10">
@@ -979,13 +979,13 @@
         </is>
       </c>
       <c r="H13">
-        <v>2.708333333333332</v>
+        <v>1.833333333333333</v>
       </c>
       <c r="I13">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J13">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="K13">
         <v>11.5</v>
@@ -1004,7 +1004,7 @@
         <v>2015</v>
       </c>
       <c r="O13">
-        <v>11.72666666666667</v>
+        <v>11.73333333333334</v>
       </c>
     </row>
     <row r="14">
@@ -1033,10 +1033,10 @@
         </is>
       </c>
       <c r="H14">
-        <v>-0.8661616161616159</v>
+        <v>-0.7555555555555571</v>
       </c>
       <c r="I14">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J14">
         <v>8</v>
@@ -1058,7 +1058,7 @@
         <v>2015</v>
       </c>
       <c r="O14">
-        <v>9.384444444444453</v>
+        <v>9.462500000000002</v>
       </c>
     </row>
     <row r="15">
@@ -1129,10 +1129,10 @@
         </is>
       </c>
       <c r="H16">
-        <v>-0.7916666666666679</v>
+        <v>-0.6944444444444458</v>
       </c>
       <c r="I16">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J16">
         <v>8.300000000000001</v>
@@ -1154,7 +1154,7 @@
         <v>2015</v>
       </c>
       <c r="O16">
-        <v>9.554444444444444</v>
+        <v>9.632142857142858</v>
       </c>
     </row>
     <row r="17">
@@ -1183,10 +1183,10 @@
         </is>
       </c>
       <c r="H17">
-        <v>-0.1785714285714288</v>
+        <v>-0.153846153846154</v>
       </c>
       <c r="I17">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J17">
         <v>6.5</v>
@@ -1208,7 +1208,7 @@
         <v>2015</v>
       </c>
       <c r="O17">
-        <v>7.711684981684986</v>
+        <v>7.828787878787876</v>
       </c>
     </row>
     <row r="18">
@@ -1237,13 +1237,13 @@
         </is>
       </c>
       <c r="H18">
-        <v>3.819940476190477</v>
+        <v>3.154761904761905</v>
       </c>
       <c r="I18">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J18">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="K18">
         <v>9.200000000000001</v>
@@ -1262,7 +1262,7 @@
         <v>2015</v>
       </c>
       <c r="O18">
-        <v>9.797500000000005</v>
+        <v>9.857142857142856</v>
       </c>
     </row>
     <row r="19">
@@ -1291,10 +1291,10 @@
         </is>
       </c>
       <c r="H19">
-        <v>-2.5</v>
+        <v>-2</v>
       </c>
       <c r="I19">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J19">
         <v>12.2</v>
@@ -1316,7 +1316,7 @@
         <v>2015</v>
       </c>
       <c r="O19">
-        <v>12.48</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="20">
@@ -1345,10 +1345,10 @@
         </is>
       </c>
       <c r="H20">
-        <v>-1.25</v>
+        <v>-1</v>
       </c>
       <c r="I20">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J20">
         <v>12.3</v>
@@ -1370,7 +1370,7 @@
         <v>2015</v>
       </c>
       <c r="O20">
-        <v>12.48</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="21">
@@ -1399,13 +1399,13 @@
         </is>
       </c>
       <c r="H21">
-        <v>-2.882440476190477</v>
+        <v>-2.476190476190476</v>
       </c>
       <c r="I21">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J21">
-        <v>9.4</v>
+        <v>9.5</v>
       </c>
       <c r="K21">
         <v>10.8</v>
@@ -1424,7 +1424,7 @@
         <v>2015</v>
       </c>
       <c r="O21">
-        <v>11.12</v>
+        <v>11.175</v>
       </c>
     </row>
     <row r="22">
@@ -1453,10 +1453,10 @@
         </is>
       </c>
       <c r="H22">
-        <v>1.354166666666666</v>
+        <v>1.249999999999999</v>
       </c>
       <c r="I22">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J22">
         <v>11.4</v>
@@ -1478,7 +1478,7 @@
         <v>2015</v>
       </c>
       <c r="O22">
-        <v>11.315</v>
+        <v>11.325</v>
       </c>
     </row>
     <row r="23">
@@ -1549,13 +1549,13 @@
         </is>
       </c>
       <c r="H24">
-        <v>-1.354166666666666</v>
+        <v>-0.6666666666666657</v>
       </c>
       <c r="I24">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J24">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="K24">
         <v>11.4</v>
@@ -1574,7 +1574,7 @@
         <v>2015</v>
       </c>
       <c r="O24">
-        <v>11.64</v>
+        <v>11.66666666666667</v>
       </c>
     </row>
     <row r="25">
@@ -1603,10 +1603,10 @@
         </is>
       </c>
       <c r="H25">
-        <v>2.083333333333332</v>
+        <v>1.833333333333333</v>
       </c>
       <c r="I25">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J25">
         <v>11.9</v>
@@ -1628,7 +1628,7 @@
         <v>2015</v>
       </c>
       <c r="O25">
-        <v>11.72666666666667</v>
+        <v>11.73333333333334</v>
       </c>
     </row>
     <row r="26">
@@ -1741,10 +1741,10 @@
         </is>
       </c>
       <c r="H28">
-        <v>-2.5</v>
+        <v>-2</v>
       </c>
       <c r="I28">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J28">
         <v>12.1</v>
@@ -1766,7 +1766,7 @@
         <v>2015</v>
       </c>
       <c r="O28">
-        <v>12.38</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="29">
@@ -1795,10 +1795,10 @@
         </is>
       </c>
       <c r="H29">
-        <v>0.5625</v>
+        <v>0.5</v>
       </c>
       <c r="I29">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J29">
         <v>10.9</v>
@@ -1820,7 +1820,7 @@
         <v>2015</v>
       </c>
       <c r="O29">
-        <v>11.04</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="30">
@@ -1852,7 +1852,7 @@
         <v>0</v>
       </c>
       <c r="I30">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J30">
         <v>10.6</v>
@@ -1874,7 +1874,7 @@
         <v>2015</v>
       </c>
       <c r="O30">
-        <v>10.96</v>
+        <v>11</v>
       </c>
     </row>
     <row r="31">
@@ -1903,10 +1903,10 @@
         </is>
       </c>
       <c r="H31">
-        <v>-0.166666666666667</v>
+        <v>-0.1428571428571431</v>
       </c>
       <c r="I31">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J31">
         <v>5.9</v>
@@ -1928,7 +1928,7 @@
         <v>2015</v>
       </c>
       <c r="O31">
-        <v>7.202380952380947</v>
+        <v>7.340018315018316</v>
       </c>
     </row>
     <row r="32">
@@ -1999,10 +1999,10 @@
         </is>
       </c>
       <c r="H33">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="I33">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J33">
         <v>12.5</v>
@@ -2024,7 +2024,7 @@
         <v>2015</v>
       </c>
       <c r="O33">
-        <v>12.48</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="34">
@@ -2095,10 +2095,10 @@
         </is>
       </c>
       <c r="H35">
-        <v>-0.625</v>
+        <v>-0.4999999999999986</v>
       </c>
       <c r="I35">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J35">
         <v>12</v>
@@ -2120,7 +2120,7 @@
         <v>2015</v>
       </c>
       <c r="O35">
-        <v>12.18</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="36">
@@ -2149,10 +2149,10 @@
         </is>
       </c>
       <c r="H36">
-        <v>1.590617715617714</v>
+        <v>1.398989898989899</v>
       </c>
       <c r="I36">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J36">
         <v>8.300000000000001</v>
@@ -2174,7 +2174,7 @@
         <v>2015</v>
       </c>
       <c r="O36">
-        <v>7.790256410256415</v>
+        <v>7.912121212121225</v>
       </c>
     </row>
     <row r="37">
@@ -2203,10 +2203,10 @@
         </is>
       </c>
       <c r="H37">
-        <v>-0.9756944444444464</v>
+        <v>-0.8472222222222229</v>
       </c>
       <c r="I37">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J37">
         <v>8.5</v>
@@ -2228,7 +2228,7 @@
         <v>2015</v>
       </c>
       <c r="O37">
-        <v>9.797500000000005</v>
+        <v>9.857142857142856</v>
       </c>
     </row>
     <row r="38">
@@ -2257,10 +2257,10 @@
         </is>
       </c>
       <c r="H38">
-        <v>0.7440476190476195</v>
+        <v>0.6666666666666664</v>
       </c>
       <c r="I38">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J38">
         <v>10.1</v>
@@ -2282,7 +2282,7 @@
         <v>2015</v>
       </c>
       <c r="O38">
-        <v>10.22285714285714</v>
+        <v>10.26666666666666</v>
       </c>
     </row>
     <row r="39">
@@ -2311,10 +2311,10 @@
         </is>
       </c>
       <c r="H39">
-        <v>-0.2386363636363633</v>
+        <v>-0.2111111111111114</v>
       </c>
       <c r="I39">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J39">
         <v>8.1</v>
@@ -2336,7 +2336,7 @@
         <v>2015</v>
       </c>
       <c r="O39">
-        <v>9.050000000000001</v>
+        <v>9.144444444444453</v>
       </c>
     </row>
     <row r="40">
@@ -2365,13 +2365,13 @@
         </is>
       </c>
       <c r="H40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I40">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J40">
-        <v>12.2</v>
+        <v>12.3</v>
       </c>
       <c r="K40">
         <v>12.2</v>
@@ -2390,7 +2390,7 @@
         <v>2015</v>
       </c>
       <c r="O40">
-        <v>12.28</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="41">
@@ -2419,13 +2419,13 @@
         </is>
       </c>
       <c r="H41">
-        <v>0.7142857142857153</v>
+        <v>0.8095238095238088</v>
       </c>
       <c r="I41">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J41">
-        <v>9.9</v>
+        <v>10</v>
       </c>
       <c r="K41">
         <v>9.5</v>
@@ -2444,7 +2444,7 @@
         <v>2015</v>
       </c>
       <c r="O41">
-        <v>10.05142857142857</v>
+        <v>10.11190476190476</v>
       </c>
     </row>
     <row r="42">
@@ -2473,10 +2473,10 @@
         </is>
       </c>
       <c r="H42">
-        <v>2.291666666666666</v>
+        <v>2</v>
       </c>
       <c r="I42">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J42">
         <v>12</v>
@@ -2498,7 +2498,7 @@
         <v>2015</v>
       </c>
       <c r="O42">
-        <v>11.79333333333333</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="43">
@@ -2527,10 +2527,10 @@
         </is>
       </c>
       <c r="H43">
-        <v>5.625</v>
+        <v>4.499999999999998</v>
       </c>
       <c r="I43">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J43">
         <v>12.5</v>
@@ -2552,7 +2552,7 @@
         <v>2015</v>
       </c>
       <c r="O43">
-        <v>12.13</v>
+        <v>12.15</v>
       </c>
     </row>
     <row r="44">
@@ -2581,10 +2581,10 @@
         </is>
       </c>
       <c r="H44">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="I44">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J44">
         <v>12.2</v>
@@ -2606,7 +2606,7 @@
         <v>2015</v>
       </c>
       <c r="O44">
-        <v>12.18</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="45">
@@ -2680,7 +2680,7 @@
         <v>0</v>
       </c>
       <c r="I46">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J46">
         <v>12.1</v>
@@ -2702,7 +2702,7 @@
         <v>2015</v>
       </c>
       <c r="O46">
-        <v>12.18</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="47">
@@ -2857,10 +2857,10 @@
         </is>
       </c>
       <c r="H50">
-        <v>0.9249387254901962</v>
+        <v>0.8065476190476198</v>
       </c>
       <c r="I50">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J50">
         <v>6.100000000000001</v>
@@ -2882,7 +2882,7 @@
         <v>2015</v>
       </c>
       <c r="O50">
-        <v>6.190073529411758</v>
+        <v>6.358630952380961</v>
       </c>
     </row>
     <row r="51">
@@ -2911,10 +2911,10 @@
         </is>
       </c>
       <c r="H51">
-        <v>4.375</v>
+        <v>3.499999999999999</v>
       </c>
       <c r="I51">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J51">
         <v>12.4</v>
@@ -2936,7 +2936,7 @@
         <v>2015</v>
       </c>
       <c r="O51">
-        <v>12.13</v>
+        <v>12.15</v>
       </c>
     </row>
     <row r="52">
@@ -3007,13 +3007,13 @@
         </is>
       </c>
       <c r="H53">
-        <v>-2.604166666666664</v>
+        <v>-1.999999999999999</v>
       </c>
       <c r="I53">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J53">
-        <v>11.2</v>
+        <v>11.3</v>
       </c>
       <c r="K53">
         <v>11.8</v>
@@ -3032,7 +3032,7 @@
         <v>2015</v>
       </c>
       <c r="O53">
-        <v>11.96</v>
+        <v>12</v>
       </c>
     </row>
     <row r="54">
@@ -3061,13 +3061,13 @@
         </is>
       </c>
       <c r="H54">
-        <v>0.625</v>
+        <v>0.9999999999999986</v>
       </c>
       <c r="I54">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J54">
-        <v>12</v>
+        <v>12.1</v>
       </c>
       <c r="K54">
         <v>11.9</v>
@@ -3086,7 +3086,7 @@
         <v>2015</v>
       </c>
       <c r="O54">
-        <v>12.06</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="55">
@@ -3118,7 +3118,7 @@
         <v>0</v>
       </c>
       <c r="I55">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J55">
         <v>11.9</v>
@@ -3140,7 +3140,7 @@
         <v>2015</v>
       </c>
       <c r="O55">
-        <v>12.06</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="56">
@@ -3169,13 +3169,13 @@
         </is>
       </c>
       <c r="H56">
-        <v>2.636904761904762</v>
+        <v>2.583333333333333</v>
       </c>
       <c r="I56">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J56">
-        <v>11</v>
+        <v>11.1</v>
       </c>
       <c r="K56">
         <v>9.9</v>
@@ -3194,7 +3194,7 @@
         <v>2015</v>
       </c>
       <c r="O56">
-        <v>10.39428571428572</v>
+        <v>10.43333333333334</v>
       </c>
     </row>
     <row r="57">
@@ -3226,7 +3226,7 @@
         <v>0</v>
       </c>
       <c r="I57">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J57">
         <v>7.4</v>
@@ -3248,7 +3248,7 @@
         <v>2015</v>
       </c>
       <c r="O57">
-        <v>8.29545454545455</v>
+        <v>8.404545454545458</v>
       </c>
     </row>
     <row r="58">
@@ -3361,10 +3361,10 @@
         </is>
       </c>
       <c r="H60">
-        <v>0.5587121212121202</v>
+        <v>0.4909090909090906</v>
       </c>
       <c r="I60">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J60">
         <v>8.1</v>
@@ -3386,7 +3386,7 @@
         <v>2015</v>
       </c>
       <c r="O60">
-        <v>8.462121212121223</v>
+        <v>8.568181818181818</v>
       </c>
     </row>
     <row r="61">
@@ -3457,13 +3457,13 @@
         </is>
       </c>
       <c r="H62">
-        <v>9.479166666666664</v>
+        <v>6.83333333333333</v>
       </c>
       <c r="I62">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J62">
-        <v>12.5</v>
+        <v>12.4</v>
       </c>
       <c r="K62">
         <v>11.2</v>
@@ -3482,7 +3482,7 @@
         <v>2015</v>
       </c>
       <c r="O62">
-        <v>11.465</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="63">
@@ -3556,7 +3556,7 @@
         <v>0</v>
       </c>
       <c r="I64">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J64">
         <v>9.9</v>
@@ -3578,7 +3578,7 @@
         <v>2015</v>
       </c>
       <c r="O64">
-        <v>10.39428571428572</v>
+        <v>10.43333333333334</v>
       </c>
     </row>
     <row r="65">
@@ -3610,7 +3610,7 @@
         <v>0</v>
       </c>
       <c r="I65">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J65">
         <v>8.4</v>
@@ -3632,7 +3632,7 @@
         <v>2015</v>
       </c>
       <c r="O65">
-        <v>9.135555555555548</v>
+        <v>9.22916666666667</v>
       </c>
     </row>
     <row r="66">
@@ -3745,10 +3745,10 @@
         </is>
       </c>
       <c r="H68">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="I68">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J68">
         <v>10.8</v>
@@ -3770,7 +3770,7 @@
         <v>2015</v>
       </c>
       <c r="O68">
-        <v>10.8</v>
+        <v>10.84</v>
       </c>
     </row>
     <row r="69">
@@ -3841,10 +3841,10 @@
         </is>
       </c>
       <c r="H70">
-        <v>0.967365967365966</v>
+        <v>0.8545454545454543</v>
       </c>
       <c r="I70">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J70">
         <v>8.1</v>
@@ -3866,7 +3866,7 @@
         <v>2015</v>
       </c>
       <c r="O70">
-        <v>8.128717948717949</v>
+        <v>8.240909090909096</v>
       </c>
     </row>
     <row r="71">
@@ -3895,10 +3895,10 @@
         </is>
       </c>
       <c r="H71">
-        <v>2.761002886002888</v>
+        <v>2.451984126984128</v>
       </c>
       <c r="I71">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J71">
         <v>9.9</v>
@@ -3920,7 +3920,7 @@
         <v>2015</v>
       </c>
       <c r="O71">
-        <v>8.796363636363628</v>
+        <v>8.895555555555548</v>
       </c>
     </row>
     <row r="72">
@@ -3949,10 +3949,10 @@
         </is>
       </c>
       <c r="H72">
-        <v>-0.3409090909090904</v>
+        <v>-0.3</v>
       </c>
       <c r="I72">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J72">
         <v>7.7</v>
@@ -3974,7 +3974,7 @@
         <v>2015</v>
       </c>
       <c r="O72">
-        <v>8.796363636363628</v>
+        <v>8.895555555555548</v>
       </c>
     </row>
     <row r="73">
@@ -4003,10 +4003,10 @@
         </is>
       </c>
       <c r="H73">
-        <v>0.06578947368421062</v>
+        <v>0.05555555555555554</v>
       </c>
       <c r="I73">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J73">
         <v>4.3</v>
@@ -4028,7 +4028,7 @@
         <v>2015</v>
       </c>
       <c r="O73">
-        <v>5.596546267629856</v>
+        <v>5.793790849673214</v>
       </c>
     </row>
     <row r="74">
@@ -4099,10 +4099,10 @@
         </is>
       </c>
       <c r="H75">
-        <v>-2.5</v>
+        <v>-2</v>
       </c>
       <c r="I75">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J75">
         <v>12.1</v>
@@ -4124,7 +4124,7 @@
         <v>2015</v>
       </c>
       <c r="O75">
-        <v>12.38</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="76">
@@ -4153,10 +4153,10 @@
         </is>
       </c>
       <c r="H76">
-        <v>-0.8482142857142865</v>
+        <v>-0.7619047619047621</v>
       </c>
       <c r="I76">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J76">
         <v>9.300000000000001</v>
@@ -4178,7 +4178,7 @@
         <v>2015</v>
       </c>
       <c r="O76">
-        <v>10.30857142857143</v>
+        <v>10.35</v>
       </c>
     </row>
     <row r="77">
@@ -4207,10 +4207,10 @@
         </is>
       </c>
       <c r="H77">
-        <v>-3.61904761904762</v>
+        <v>-3.249999999999999</v>
       </c>
       <c r="I77">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J77">
         <v>9.700000000000001</v>
@@ -4232,7 +4232,7 @@
         <v>2015</v>
       </c>
       <c r="O77">
-        <v>11.465</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="78">
@@ -4303,10 +4303,10 @@
         </is>
       </c>
       <c r="H79">
-        <v>-1.005050505050505</v>
+        <v>-0.8805555555555571</v>
       </c>
       <c r="I79">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J79">
         <v>8</v>
@@ -4328,7 +4328,7 @@
         <v>2015</v>
       </c>
       <c r="O79">
-        <v>9.47333333333334</v>
+        <v>9.550000000000001</v>
       </c>
     </row>
     <row r="80">
@@ -4402,7 +4402,7 @@
         <v>0</v>
       </c>
       <c r="I81">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J81">
         <v>11.5</v>
@@ -4424,7 +4424,7 @@
         <v>2015</v>
       </c>
       <c r="O81">
-        <v>11.72666666666667</v>
+        <v>11.73333333333334</v>
       </c>
     </row>
     <row r="82">
@@ -4453,10 +4453,10 @@
         </is>
       </c>
       <c r="H82">
-        <v>-3.75</v>
+        <v>-3</v>
       </c>
       <c r="I82">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J82">
         <v>12.1</v>
@@ -4478,7 +4478,7 @@
         <v>2015</v>
       </c>
       <c r="O82">
-        <v>12.48</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="83">
@@ -4507,13 +4507,13 @@
         </is>
       </c>
       <c r="H83">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I83">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J83">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="K83">
         <v>11.9</v>
@@ -4532,7 +4532,7 @@
         <v>2015</v>
       </c>
       <c r="O83">
-        <v>12.06</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="84">
@@ -4561,10 +4561,10 @@
         </is>
       </c>
       <c r="H84">
-        <v>1.25</v>
+        <v>1.083333333333333</v>
       </c>
       <c r="I84">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J84">
         <v>11.2</v>
@@ -4586,7 +4586,7 @@
         <v>2015</v>
       </c>
       <c r="O84">
-        <v>11.12</v>
+        <v>11.175</v>
       </c>
     </row>
     <row r="85">
@@ -4657,10 +4657,10 @@
         </is>
       </c>
       <c r="H86">
-        <v>3.541666666666664</v>
+        <v>2.999999999999999</v>
       </c>
       <c r="I86">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J86">
         <v>12</v>
@@ -4682,7 +4682,7 @@
         <v>2015</v>
       </c>
       <c r="O86">
-        <v>11.54</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="87">
@@ -4711,10 +4711,10 @@
         </is>
       </c>
       <c r="H87">
-        <v>1.855158730158733</v>
+        <v>1.640873015873016</v>
       </c>
       <c r="I87">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J87">
         <v>9.800000000000001</v>
@@ -4736,7 +4736,7 @@
         <v>2015</v>
       </c>
       <c r="O87">
-        <v>9.295555555555548</v>
+        <v>9.384722222222221</v>
       </c>
     </row>
     <row r="88">
@@ -4765,10 +4765,10 @@
         </is>
       </c>
       <c r="H88">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="I88">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J88">
         <v>12.5</v>
@@ -4790,7 +4790,7 @@
         <v>2015</v>
       </c>
       <c r="O88">
-        <v>12.48</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="89">
@@ -4903,10 +4903,10 @@
         </is>
       </c>
       <c r="H91">
-        <v>-0.625</v>
+        <v>-0.5833333333333328</v>
       </c>
       <c r="I91">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J91">
         <v>11</v>
@@ -4928,7 +4928,7 @@
         <v>2015</v>
       </c>
       <c r="O91">
-        <v>11.465</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="92">
@@ -4957,10 +4957,10 @@
         </is>
       </c>
       <c r="H92">
-        <v>1.874999999999998</v>
+        <v>1.666666666666666</v>
       </c>
       <c r="I92">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J92">
         <v>11.8</v>
@@ -4982,7 +4982,7 @@
         <v>2015</v>
       </c>
       <c r="O92">
-        <v>11.64</v>
+        <v>11.66666666666667</v>
       </c>
     </row>
     <row r="93">
@@ -5053,10 +5053,10 @@
         </is>
       </c>
       <c r="H94">
-        <v>-2.5</v>
+        <v>-1.999999999999999</v>
       </c>
       <c r="I94">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J94">
         <v>11.7</v>
@@ -5078,7 +5078,7 @@
         <v>2015</v>
       </c>
       <c r="O94">
-        <v>12.18</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="95">
@@ -5107,13 +5107,13 @@
         </is>
       </c>
       <c r="H95">
-        <v>2.083333333333332</v>
+        <v>2.333333333333333</v>
       </c>
       <c r="I95">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J95">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="K95">
         <v>11.5</v>
@@ -5132,7 +5132,7 @@
         <v>2015</v>
       </c>
       <c r="O95">
-        <v>11.72666666666667</v>
+        <v>11.73333333333334</v>
       </c>
     </row>
     <row r="96">
@@ -5161,10 +5161,10 @@
         </is>
       </c>
       <c r="H96">
-        <v>3.854166666666664</v>
+        <v>3.333333333333331</v>
       </c>
       <c r="I96">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J96">
         <v>12</v>
@@ -5186,7 +5186,7 @@
         <v>2015</v>
       </c>
       <c r="O96">
-        <v>11.465</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="97">
@@ -5215,13 +5215,13 @@
         </is>
       </c>
       <c r="H97">
-        <v>-1.220238095238097</v>
+        <v>-0.9464285714285723</v>
       </c>
       <c r="I97">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J97">
-        <v>8.800000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="K97">
         <v>9.600000000000001</v>
@@ -5240,7 +5240,7 @@
         <v>2015</v>
       </c>
       <c r="O97">
-        <v>10.13714285714286</v>
+        <v>10.18333333333334</v>
       </c>
     </row>
     <row r="98">
@@ -5269,10 +5269,10 @@
         </is>
       </c>
       <c r="H98">
-        <v>1.874999999999998</v>
+        <v>1.666666666666664</v>
       </c>
       <c r="I98">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J98">
         <v>11.6</v>
@@ -5294,7 +5294,7 @@
         <v>2015</v>
       </c>
       <c r="O98">
-        <v>11.39</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="99">
@@ -5407,10 +5407,10 @@
         </is>
       </c>
       <c r="H101">
-        <v>-6.044642857142855</v>
+        <v>-5.416666666666664</v>
       </c>
       <c r="I101">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J101">
         <v>9.800000000000001</v>
@@ -5432,7 +5432,7 @@
         <v>2015</v>
       </c>
       <c r="O101">
-        <v>11.96</v>
+        <v>12</v>
       </c>
     </row>
     <row r="102">
@@ -5461,10 +5461,10 @@
         </is>
       </c>
       <c r="H102">
-        <v>0.3869047619047619</v>
+        <v>0.3333333333333336</v>
       </c>
       <c r="I102">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J102">
         <v>10.1</v>
@@ -5486,7 +5486,7 @@
         <v>2015</v>
       </c>
       <c r="O102">
-        <v>10.39428571428572</v>
+        <v>10.43333333333334</v>
       </c>
     </row>
     <row r="103">
@@ -5515,13 +5515,13 @@
         </is>
       </c>
       <c r="H103">
-        <v>0</v>
+        <v>0.1111111111111114</v>
       </c>
       <c r="I103">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J103">
-        <v>8.6</v>
+        <v>8.700000000000001</v>
       </c>
       <c r="K103">
         <v>8.6</v>
@@ -5540,7 +5540,7 @@
         <v>2015</v>
       </c>
       <c r="O103">
-        <v>9.295555555555548</v>
+        <v>9.384722222222221</v>
       </c>
     </row>
     <row r="104">
@@ -5569,10 +5569,10 @@
         </is>
       </c>
       <c r="H104">
-        <v>-1.865079365079366</v>
+        <v>-1.654761904761905</v>
       </c>
       <c r="I104">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J104">
         <v>9</v>
@@ -5594,7 +5594,7 @@
         <v>2015</v>
       </c>
       <c r="O104">
-        <v>10.55</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="105">
@@ -5623,10 +5623,10 @@
         </is>
       </c>
       <c r="H105">
-        <v>0.4166666666666661</v>
+        <v>0.5</v>
       </c>
       <c r="I105">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J105">
         <v>11.7</v>
@@ -5648,7 +5648,7 @@
         <v>2015</v>
       </c>
       <c r="O105">
-        <v>11.79333333333333</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="106">
@@ -5719,10 +5719,10 @@
         </is>
       </c>
       <c r="H107">
-        <v>3.854166666666664</v>
+        <v>3.333333333333331</v>
       </c>
       <c r="I107">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J107">
         <v>12</v>
@@ -5744,7 +5744,7 @@
         <v>2015</v>
       </c>
       <c r="O107">
-        <v>11.465</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="108">
@@ -5773,10 +5773,10 @@
         </is>
       </c>
       <c r="H108">
-        <v>-2.355158730158733</v>
+        <v>-2.085317460317462</v>
       </c>
       <c r="I108">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J108">
         <v>8.200000000000001</v>
@@ -5798,7 +5798,7 @@
         <v>2015</v>
       </c>
       <c r="O108">
-        <v>10.30857142857143</v>
+        <v>10.35</v>
       </c>
     </row>
     <row r="109">
@@ -5869,10 +5869,10 @@
         </is>
       </c>
       <c r="H110">
-        <v>3.75</v>
+        <v>3</v>
       </c>
       <c r="I110">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J110">
         <v>12.5</v>
@@ -5894,7 +5894,7 @@
         <v>2015</v>
       </c>
       <c r="O110">
-        <v>12.28</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="111">
@@ -5965,13 +5965,13 @@
         </is>
       </c>
       <c r="H112">
-        <v>-2.916666666666664</v>
+        <v>-2.333333333333331</v>
       </c>
       <c r="I112">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J112">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="K112">
         <v>11.8</v>
@@ -5990,7 +5990,7 @@
         <v>2015</v>
       </c>
       <c r="O112">
-        <v>11.96</v>
+        <v>12</v>
       </c>
     </row>
     <row r="113">
@@ -6019,10 +6019,10 @@
         </is>
       </c>
       <c r="H113">
-        <v>5.229166666666664</v>
+        <v>4.616666666666664</v>
       </c>
       <c r="I113">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J113">
         <v>11.9</v>
@@ -6044,7 +6044,7 @@
         <v>2015</v>
       </c>
       <c r="O113">
-        <v>10.88</v>
+        <v>10.92</v>
       </c>
     </row>
     <row r="114">
@@ -6157,13 +6157,13 @@
         </is>
       </c>
       <c r="H116">
-        <v>-1.62058080808081</v>
+        <v>-1.3234126984127</v>
       </c>
       <c r="I116">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J116">
-        <v>8.1</v>
+        <v>8.200000000000001</v>
       </c>
       <c r="K116">
         <v>9.300000000000001</v>
@@ -6182,7 +6182,7 @@
         <v>2015</v>
       </c>
       <c r="O116">
-        <v>9.884999999999998</v>
+        <v>9.942857142857145</v>
       </c>
     </row>
     <row r="117">
@@ -6211,13 +6211,13 @@
         </is>
       </c>
       <c r="H117">
-        <v>2.645833333333332</v>
+        <v>1.999999999999999</v>
       </c>
       <c r="I117">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J117">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="K117">
         <v>10.7</v>
@@ -6236,7 +6236,7 @@
         <v>2015</v>
       </c>
       <c r="O117">
-        <v>11.04</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="118">
@@ -6265,10 +6265,10 @@
         </is>
       </c>
       <c r="H118">
-        <v>-1.041666666666666</v>
+        <v>-1</v>
       </c>
       <c r="I118">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J118">
         <v>11.6</v>
@@ -6290,7 +6290,7 @@
         <v>2015</v>
       </c>
       <c r="O118">
-        <v>11.96</v>
+        <v>12</v>
       </c>
     </row>
     <row r="119">
@@ -6319,10 +6319,10 @@
         </is>
       </c>
       <c r="H119">
-        <v>7.916666666666664</v>
+        <v>6.499999999999997</v>
       </c>
       <c r="I119">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J119">
         <v>12.4</v>
@@ -6344,7 +6344,7 @@
         <v>2015</v>
       </c>
       <c r="O119">
-        <v>11.54</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="120">
@@ -6373,10 +6373,10 @@
         </is>
       </c>
       <c r="H120">
-        <v>2.916666666666664</v>
+        <v>2.666666666666664</v>
       </c>
       <c r="I120">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J120">
         <v>11.8</v>
@@ -6398,7 +6398,7 @@
         <v>2015</v>
       </c>
       <c r="O120">
-        <v>11.39</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="121">
@@ -6427,10 +6427,10 @@
         </is>
       </c>
       <c r="H121">
-        <v>0.08333333333333348</v>
+        <v>0.07692307692307701</v>
       </c>
       <c r="I121">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J121">
         <v>6.300000000000001</v>
@@ -6452,7 +6452,7 @@
         <v>2015</v>
       </c>
       <c r="O121">
-        <v>7.28904761904763</v>
+        <v>7.418589743589744</v>
       </c>
     </row>
     <row r="122">
@@ -6523,10 +6523,10 @@
         </is>
       </c>
       <c r="H123">
-        <v>2.11904761904762</v>
+        <v>1.916666666666667</v>
       </c>
       <c r="I123">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J123">
         <v>10.7</v>
@@ -6548,7 +6548,7 @@
         <v>2015</v>
       </c>
       <c r="O123">
-        <v>10.22285714285714</v>
+        <v>10.26666666666666</v>
       </c>
     </row>
     <row r="124">
@@ -6619,13 +6619,13 @@
         </is>
       </c>
       <c r="H125">
-        <v>-3.125</v>
+        <v>-1.999999999999999</v>
       </c>
       <c r="I125">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J125">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="K125">
         <v>12.2</v>
@@ -6644,7 +6644,7 @@
         <v>2015</v>
       </c>
       <c r="O125">
-        <v>12.28</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="126">
@@ -6673,10 +6673,10 @@
         </is>
       </c>
       <c r="H126">
-        <v>-1.143939393939394</v>
+        <v>-1.005555555555557</v>
       </c>
       <c r="I126">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J126">
         <v>8</v>
@@ -6698,7 +6698,7 @@
         <v>2015</v>
       </c>
       <c r="O126">
-        <v>9.554444444444444</v>
+        <v>9.632142857142858</v>
       </c>
     </row>
     <row r="127">
@@ -6727,10 +6727,10 @@
         </is>
       </c>
       <c r="H127">
-        <v>-0.208333333333333</v>
+        <v>-0.181818181818182</v>
       </c>
       <c r="I127">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J127">
         <v>7.300000000000001</v>
@@ -6752,7 +6752,7 @@
         <v>2015</v>
       </c>
       <c r="O127">
-        <v>8.378787878787875</v>
+        <v>8.486363636363627</v>
       </c>
     </row>
     <row r="128">
@@ -6781,13 +6781,13 @@
         </is>
       </c>
       <c r="H128">
-        <v>-2.5</v>
+        <v>-1.499999999999999</v>
       </c>
       <c r="I128">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J128">
-        <v>11.7</v>
+        <v>11.8</v>
       </c>
       <c r="K128">
         <v>12.1</v>
@@ -6806,7 +6806,7 @@
         <v>2015</v>
       </c>
       <c r="O128">
-        <v>12.18</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="129">
@@ -6835,10 +6835,10 @@
         </is>
       </c>
       <c r="H129">
-        <v>0.3125</v>
+        <v>0.2857142857142861</v>
       </c>
       <c r="I129">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J129">
         <v>9.5</v>
@@ -6860,7 +6860,7 @@
         <v>2015</v>
       </c>
       <c r="O129">
-        <v>9.884999999999998</v>
+        <v>9.942857142857145</v>
       </c>
     </row>
     <row r="130">
@@ -6889,10 +6889,10 @@
         </is>
       </c>
       <c r="H130">
-        <v>-0.9583333333333339</v>
+        <v>-0.85</v>
       </c>
       <c r="I130">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J130">
         <v>10.3</v>
@@ -6914,7 +6914,7 @@
         <v>2015</v>
       </c>
       <c r="O130">
-        <v>11.04</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="131">
@@ -6985,10 +6985,10 @@
         </is>
       </c>
       <c r="H132">
-        <v>0.1470588235294117</v>
+        <v>0.1291666666666666</v>
       </c>
       <c r="I132">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J132">
         <v>5.300000000000001</v>
@@ -7010,7 +7010,7 @@
         <v>2015</v>
       </c>
       <c r="O132">
-        <v>6.36210784313726</v>
+        <v>6.521130952380942</v>
       </c>
     </row>
     <row r="133">
@@ -7039,13 +7039,13 @@
         </is>
       </c>
       <c r="H133">
-        <v>0.5902777777777786</v>
+        <v>0.375</v>
       </c>
       <c r="I133">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J133">
-        <v>9.300000000000001</v>
+        <v>9.200000000000001</v>
       </c>
       <c r="K133">
         <v>8.9</v>
@@ -7064,7 +7064,7 @@
         <v>2015</v>
       </c>
       <c r="O133">
-        <v>9.554444444444444</v>
+        <v>9.632142857142858</v>
       </c>
     </row>
     <row r="134">
@@ -7093,10 +7093,10 @@
         </is>
       </c>
       <c r="H134">
-        <v>-2.479166666666666</v>
+        <v>-2.249999999999999</v>
       </c>
       <c r="I134">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J134">
         <v>10.6</v>
@@ -7118,7 +7118,7 @@
         <v>2015</v>
       </c>
       <c r="O134">
-        <v>11.64</v>
+        <v>11.66666666666667</v>
       </c>
     </row>
     <row r="135">
@@ -7231,10 +7231,10 @@
         </is>
       </c>
       <c r="H137">
-        <v>2.666666666666667</v>
+        <v>2.383333333333333</v>
       </c>
       <c r="I137">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J137">
         <v>11.2</v>
@@ -7256,7 +7256,7 @@
         <v>2015</v>
       </c>
       <c r="O137">
-        <v>10.63333333333334</v>
+        <v>10.68</v>
       </c>
     </row>
     <row r="138">
@@ -7285,13 +7285,13 @@
         </is>
       </c>
       <c r="H138">
-        <v>3.729166666666664</v>
+        <v>2.916666666666664</v>
       </c>
       <c r="I138">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J138">
-        <v>11.7</v>
+        <v>11.6</v>
       </c>
       <c r="K138">
         <v>10.6</v>
@@ -7310,7 +7310,7 @@
         <v>2015</v>
       </c>
       <c r="O138">
-        <v>10.96</v>
+        <v>11</v>
       </c>
     </row>
     <row r="139">
@@ -7381,10 +7381,10 @@
         </is>
       </c>
       <c r="H140">
-        <v>-4.791666666666664</v>
+        <v>-4.166666666666663</v>
       </c>
       <c r="I140">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J140">
         <v>11.1</v>
@@ -7406,7 +7406,7 @@
         <v>2015</v>
       </c>
       <c r="O140">
-        <v>12.18</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="141">
@@ -7435,13 +7435,13 @@
         </is>
       </c>
       <c r="H141">
-        <v>1.194444444444446</v>
+        <v>1.609126984126986</v>
       </c>
       <c r="I141">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J141">
-        <v>9.1</v>
+        <v>9.5</v>
       </c>
       <c r="K141">
         <v>8.200000000000001</v>
@@ -7460,7 +7460,7 @@
         <v>2015</v>
       </c>
       <c r="O141">
-        <v>8.960000000000008</v>
+        <v>9.055555555555546</v>
       </c>
     </row>
     <row r="142">
@@ -7492,7 +7492,7 @@
         <v>0</v>
       </c>
       <c r="I142">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J142">
         <v>11</v>
@@ -7514,7 +7514,7 @@
         <v>2015</v>
       </c>
       <c r="O142">
-        <v>11.315</v>
+        <v>11.325</v>
       </c>
     </row>
     <row r="143">
@@ -7588,7 +7588,7 @@
         <v>0</v>
       </c>
       <c r="I144">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J144">
         <v>11.1</v>
@@ -7610,7 +7610,7 @@
         <v>2015</v>
       </c>
       <c r="O144">
-        <v>11.39</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="145">
@@ -7639,10 +7639,10 @@
         </is>
       </c>
       <c r="H145">
-        <v>8.098214285714285</v>
+        <v>7.083333333333329</v>
       </c>
       <c r="I145">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J145">
         <v>12.1</v>
@@ -7664,7 +7664,7 @@
         <v>2015</v>
       </c>
       <c r="O145">
-        <v>10.22285714285714</v>
+        <v>10.26666666666666</v>
       </c>
     </row>
     <row r="146">
@@ -7693,10 +7693,10 @@
         </is>
       </c>
       <c r="H146">
-        <v>-1.894841269841272</v>
+        <v>-1.696428571428572</v>
       </c>
       <c r="I146">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J146">
         <v>8.700000000000001</v>
@@ -7718,7 +7718,7 @@
         <v>2015</v>
       </c>
       <c r="O146">
-        <v>10.39428571428572</v>
+        <v>10.43333333333334</v>
       </c>
     </row>
     <row r="147">
@@ -7789,13 +7789,13 @@
         </is>
       </c>
       <c r="H148">
-        <v>-2.499999999999998</v>
+        <v>-2.416666666666664</v>
       </c>
       <c r="I148">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J148">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="K148">
         <v>11.6</v>
@@ -7814,7 +7814,7 @@
         <v>2015</v>
       </c>
       <c r="O148">
-        <v>11.79333333333333</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="149">
@@ -7885,10 +7885,10 @@
         </is>
       </c>
       <c r="H150">
-        <v>-3.562499999999998</v>
+        <v>-3.116666666666664</v>
       </c>
       <c r="I150">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J150">
         <v>10.5</v>
@@ -7910,7 +7910,7 @@
         <v>2015</v>
       </c>
       <c r="O150">
-        <v>11.79333333333333</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="151">
@@ -7939,10 +7939,10 @@
         </is>
       </c>
       <c r="H151">
-        <v>0.7291666666666661</v>
+        <v>0.6666666666666657</v>
       </c>
       <c r="I151">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J151">
         <v>11.4</v>
@@ -7964,7 +7964,7 @@
         <v>2015</v>
       </c>
       <c r="O151">
-        <v>11.465</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="152">
@@ -7993,10 +7993,10 @@
         </is>
       </c>
       <c r="H152">
-        <v>-5.416666666666666</v>
+        <v>-4.499999999999998</v>
       </c>
       <c r="I152">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J152">
         <v>11.6</v>
@@ -8018,7 +8018,7 @@
         <v>2015</v>
       </c>
       <c r="O152">
-        <v>12.38</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="153">
@@ -8047,10 +8047,10 @@
         </is>
       </c>
       <c r="H153">
-        <v>-3.479166666666664</v>
+        <v>-3.166666666666664</v>
       </c>
       <c r="I153">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J153">
         <v>10.7</v>
@@ -8072,7 +8072,7 @@
         <v>2015</v>
       </c>
       <c r="O153">
-        <v>11.86</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="154">
@@ -8101,10 +8101,10 @@
         </is>
       </c>
       <c r="H154">
-        <v>-6.979166666666664</v>
+        <v>-5.83333333333333</v>
       </c>
       <c r="I154">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J154">
         <v>11.2</v>
@@ -8126,7 +8126,7 @@
         <v>2015</v>
       </c>
       <c r="O154">
-        <v>12.38</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="155">
@@ -8158,10 +8158,10 @@
         <v>2.25</v>
       </c>
       <c r="I155">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J155">
-        <v>11</v>
+        <v>11.1</v>
       </c>
       <c r="K155">
         <v>10.1</v>
@@ -8180,7 +8180,7 @@
         <v>2015</v>
       </c>
       <c r="O155">
-        <v>10.55</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="156">
@@ -8209,13 +8209,13 @@
         </is>
       </c>
       <c r="H156">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="I156">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J156">
-        <v>12.4</v>
+        <v>12.5</v>
       </c>
       <c r="K156">
         <v>12.2</v>
@@ -8234,7 +8234,7 @@
         <v>2015</v>
       </c>
       <c r="O156">
-        <v>12.28</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="157">
@@ -8263,10 +8263,10 @@
         </is>
       </c>
       <c r="H157">
-        <v>-0.09615384615384626</v>
+        <v>-0.08333333333333322</v>
       </c>
       <c r="I157">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J157">
         <v>7</v>
@@ -8288,7 +8288,7 @@
         <v>2015</v>
       </c>
       <c r="O157">
-        <v>8.044102564102564</v>
+        <v>8.162121212121201</v>
       </c>
     </row>
     <row r="158">
@@ -8317,10 +8317,10 @@
         </is>
       </c>
       <c r="H158">
-        <v>0.3124999999999996</v>
+        <v>0.2727272727272723</v>
       </c>
       <c r="I158">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J158">
         <v>7.7</v>
@@ -8342,7 +8342,7 @@
         <v>2015</v>
       </c>
       <c r="O158">
-        <v>8.29545454545455</v>
+        <v>8.404545454545458</v>
       </c>
     </row>
     <row r="159">
@@ -8413,13 +8413,13 @@
         </is>
       </c>
       <c r="H160">
-        <v>-1.833333333333334</v>
+        <v>-1.4</v>
       </c>
       <c r="I160">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J160">
-        <v>10.3</v>
+        <v>10.4</v>
       </c>
       <c r="K160">
         <v>11</v>
@@ -8438,7 +8438,7 @@
         <v>2015</v>
       </c>
       <c r="O160">
-        <v>11.315</v>
+        <v>11.325</v>
       </c>
     </row>
     <row r="161">
@@ -8467,10 +8467,10 @@
         </is>
       </c>
       <c r="H161">
-        <v>3.034271284271287</v>
+        <v>2.685317460317462</v>
       </c>
       <c r="I161">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J161">
         <v>10.1</v>
@@ -8492,7 +8492,7 @@
         <v>2015</v>
       </c>
       <c r="O161">
-        <v>8.878181818181817</v>
+        <v>8.975555555555548</v>
       </c>
     </row>
     <row r="162">
@@ -8521,10 +8521,10 @@
         </is>
       </c>
       <c r="H162">
-        <v>-2.636904761904762</v>
+        <v>-2.333333333333333</v>
       </c>
       <c r="I162">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J162">
         <v>9.9</v>
@@ -8546,7 +8546,7 @@
         <v>2015</v>
       </c>
       <c r="O162">
-        <v>11.315</v>
+        <v>11.325</v>
       </c>
     </row>
     <row r="163">
@@ -8575,13 +8575,13 @@
         </is>
       </c>
       <c r="H163">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I163">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J163">
-        <v>10.5</v>
+        <v>10.6</v>
       </c>
       <c r="K163">
         <v>10.5</v>
@@ -8600,7 +8600,7 @@
         <v>2015</v>
       </c>
       <c r="O163">
-        <v>10.88</v>
+        <v>10.92</v>
       </c>
     </row>
     <row r="164">
@@ -8671,13 +8671,13 @@
         </is>
       </c>
       <c r="H165">
-        <v>0.1470588235294117</v>
+        <v>0.0625</v>
       </c>
       <c r="I165">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J165">
-        <v>5.2</v>
+        <v>5.100000000000001</v>
       </c>
       <c r="K165">
         <v>5</v>
@@ -8696,7 +8696,7 @@
         <v>2015</v>
       </c>
       <c r="O165">
-        <v>6.278308823529417</v>
+        <v>6.439880952380954</v>
       </c>
     </row>
     <row r="166">
@@ -8725,10 +8725,10 @@
         </is>
       </c>
       <c r="H166">
-        <v>3.854166666666664</v>
+        <v>3.333333333333331</v>
       </c>
       <c r="I166">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J166">
         <v>12</v>
@@ -8750,7 +8750,7 @@
         <v>2015</v>
       </c>
       <c r="O166">
-        <v>11.465</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="167">
@@ -8779,10 +8779,10 @@
         </is>
       </c>
       <c r="H167">
-        <v>-1.299603174603176</v>
+        <v>-1.154761904761905</v>
       </c>
       <c r="I167">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J167">
         <v>9</v>
@@ -8804,7 +8804,7 @@
         <v>2015</v>
       </c>
       <c r="O167">
-        <v>10.30857142857143</v>
+        <v>10.35</v>
       </c>
     </row>
     <row r="168">
@@ -8833,10 +8833,10 @@
         </is>
       </c>
       <c r="H168">
-        <v>4.375</v>
+        <v>3.499999999999999</v>
       </c>
       <c r="I168">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J168">
         <v>12.4</v>
@@ -8858,7 +8858,7 @@
         <v>2015</v>
       </c>
       <c r="O168">
-        <v>12.13</v>
+        <v>12.15</v>
       </c>
     </row>
     <row r="169">
@@ -8971,10 +8971,10 @@
         </is>
       </c>
       <c r="H171">
-        <v>-0.8333333333333321</v>
+        <v>-0.8333333333333328</v>
       </c>
       <c r="I171">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J171">
         <v>11.5</v>
@@ -8996,7 +8996,7 @@
         <v>2015</v>
       </c>
       <c r="O171">
-        <v>11.86</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="172">
@@ -9067,13 +9067,13 @@
         </is>
       </c>
       <c r="H173">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I173">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J173">
-        <v>12.5</v>
+        <v>12.4</v>
       </c>
       <c r="K173">
         <v>12.5</v>
@@ -9118,10 +9118,10 @@
         </is>
       </c>
       <c r="H174">
-        <v>-1.046037296037295</v>
+        <v>-0.9212121212121207</v>
       </c>
       <c r="I174">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J174">
         <v>7</v>
@@ -9143,7 +9143,7 @@
         <v>2015</v>
       </c>
       <c r="O174">
-        <v>8.796363636363628</v>
+        <v>8.895555555555548</v>
       </c>
     </row>
     <row r="175">
@@ -9172,13 +9172,13 @@
         </is>
       </c>
       <c r="H175">
-        <v>7.916666666666664</v>
+        <v>4.666666666666663</v>
       </c>
       <c r="I175">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J175">
-        <v>12.3</v>
+        <v>12.1</v>
       </c>
       <c r="K175">
         <v>10.9</v>
@@ -9197,7 +9197,7 @@
         <v>2015</v>
       </c>
       <c r="O175">
-        <v>11.22</v>
+        <v>11.25</v>
       </c>
     </row>
     <row r="176">
@@ -9226,10 +9226,10 @@
         </is>
       </c>
       <c r="H176">
-        <v>0.6011904761904772</v>
+        <v>0.5219780219780226</v>
       </c>
       <c r="I176">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J176">
         <v>6.600000000000001</v>
@@ -9251,7 +9251,7 @@
         <v>2015</v>
       </c>
       <c r="O176">
-        <v>7.029047619047613</v>
+        <v>7.181318681318679</v>
       </c>
     </row>
     <row r="177">
@@ -9280,13 +9280,13 @@
         </is>
       </c>
       <c r="H177">
-        <v>2.288690476190477</v>
+        <v>1.461904761904762</v>
       </c>
       <c r="I177">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J177">
-        <v>10.5</v>
+        <v>10.2</v>
       </c>
       <c r="K177">
         <v>9.300000000000001</v>
@@ -9305,7 +9305,7 @@
         <v>2015</v>
       </c>
       <c r="O177">
-        <v>9.884999999999998</v>
+        <v>9.942857142857145</v>
       </c>
     </row>
     <row r="178">
@@ -9376,10 +9376,10 @@
         </is>
       </c>
       <c r="H179">
-        <v>-1.375</v>
+        <v>-1.25</v>
       </c>
       <c r="I179">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J179">
         <v>10.1</v>
@@ -9401,7 +9401,7 @@
         <v>2015</v>
       </c>
       <c r="O179">
-        <v>11.04</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="180">
@@ -9433,7 +9433,7 @@
         <v>0</v>
       </c>
       <c r="I180">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J180">
         <v>11.6</v>
@@ -9455,7 +9455,7 @@
         <v>2015</v>
       </c>
       <c r="O180">
-        <v>11.79333333333333</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="181">
@@ -9484,10 +9484,10 @@
         </is>
       </c>
       <c r="H181">
-        <v>1.727904040404041</v>
+        <v>1.521464646464648</v>
       </c>
       <c r="I181">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J181">
         <v>9</v>
@@ -9509,7 +9509,7 @@
         <v>2015</v>
       </c>
       <c r="O181">
-        <v>8.462121212121223</v>
+        <v>8.568181818181818</v>
       </c>
     </row>
     <row r="182">
@@ -9538,10 +9538,10 @@
         </is>
       </c>
       <c r="H182">
-        <v>3.229166666666664</v>
+        <v>2.916666666666664</v>
       </c>
       <c r="I182">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J182">
         <v>11.8</v>
@@ -9563,7 +9563,7 @@
         <v>2015</v>
       </c>
       <c r="O182">
-        <v>11.315</v>
+        <v>11.325</v>
       </c>
     </row>
     <row r="183">
@@ -9592,10 +9592,10 @@
         </is>
       </c>
       <c r="H183">
-        <v>-3.395833333333333</v>
+        <v>-3.083333333333333</v>
       </c>
       <c r="I183">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J183">
         <v>10</v>
@@ -9617,7 +9617,7 @@
         <v>2015</v>
       </c>
       <c r="O183">
-        <v>11.54</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="184">
@@ -9646,10 +9646,10 @@
         </is>
       </c>
       <c r="H184">
-        <v>1.874999999999998</v>
+        <v>1.666666666666666</v>
       </c>
       <c r="I184">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J184">
         <v>11.8</v>
@@ -9671,7 +9671,7 @@
         <v>2015</v>
       </c>
       <c r="O184">
-        <v>11.64</v>
+        <v>11.66666666666667</v>
       </c>
     </row>
     <row r="185">
@@ -9742,13 +9742,13 @@
         </is>
       </c>
       <c r="H186">
-        <v>3.312499999999998</v>
+        <v>1.25</v>
       </c>
       <c r="I186">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J186">
-        <v>11.6</v>
+        <v>11.1</v>
       </c>
       <c r="K186">
         <v>10.6</v>
@@ -9767,7 +9767,7 @@
         <v>2015</v>
       </c>
       <c r="O186">
-        <v>10.96</v>
+        <v>11</v>
       </c>
     </row>
     <row r="187">
@@ -9796,10 +9796,10 @@
         </is>
       </c>
       <c r="H187">
-        <v>0.5587121212121202</v>
+        <v>0.4909090909090906</v>
       </c>
       <c r="I187">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J187">
         <v>8.1</v>
@@ -9821,7 +9821,7 @@
         <v>2015</v>
       </c>
       <c r="O187">
-        <v>8.462121212121223</v>
+        <v>8.568181818181818</v>
       </c>
     </row>
     <row r="188">
@@ -9850,10 +9850,10 @@
         </is>
       </c>
       <c r="H188">
-        <v>-0.8854166666666679</v>
+        <v>-0.7857142857142861</v>
       </c>
       <c r="I188">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J188">
         <v>8.800000000000001</v>
@@ -9875,7 +9875,7 @@
         <v>2015</v>
       </c>
       <c r="O188">
-        <v>9.9725</v>
+        <v>10.02857142857142</v>
       </c>
     </row>
     <row r="189">
@@ -9904,10 +9904,10 @@
         </is>
       </c>
       <c r="H189">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="I189">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J189">
         <v>12.5</v>
@@ -9929,7 +9929,7 @@
         <v>2015</v>
       </c>
       <c r="O189">
-        <v>12.48</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="190">
@@ -10042,10 +10042,10 @@
         </is>
       </c>
       <c r="H192">
-        <v>4.166666666666666</v>
+        <v>3.499999999999999</v>
       </c>
       <c r="I192">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J192">
         <v>12.2</v>
@@ -10067,7 +10067,7 @@
         <v>2015</v>
       </c>
       <c r="O192">
-        <v>11.79333333333333</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="193">
@@ -10096,10 +10096,10 @@
         </is>
       </c>
       <c r="H193">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="I193">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J193">
         <v>12.5</v>
@@ -10121,7 +10121,7 @@
         <v>2015</v>
       </c>
       <c r="O193">
-        <v>12.38</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="194">
@@ -10150,10 +10150,10 @@
         </is>
       </c>
       <c r="H194">
-        <v>3.749999999999998</v>
+        <v>3.166666666666664</v>
       </c>
       <c r="I194">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J194">
         <v>12.1</v>
@@ -10175,7 +10175,7 @@
         <v>2015</v>
       </c>
       <c r="O194">
-        <v>11.64</v>
+        <v>11.66666666666667</v>
       </c>
     </row>
     <row r="195">
@@ -10204,10 +10204,10 @@
         </is>
       </c>
       <c r="H195">
-        <v>-5.062499999999997</v>
+        <v>-4.583333333333331</v>
       </c>
       <c r="I195">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J195">
         <v>10</v>
@@ -10229,7 +10229,7 @@
         <v>2015</v>
       </c>
       <c r="O195">
-        <v>11.86</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="196">
@@ -10258,10 +10258,10 @@
         </is>
       </c>
       <c r="H196">
-        <v>2.708333333333332</v>
+        <v>2.333333333333333</v>
       </c>
       <c r="I196">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J196">
         <v>12</v>
@@ -10283,7 +10283,7 @@
         <v>2015</v>
       </c>
       <c r="O196">
-        <v>11.72666666666667</v>
+        <v>11.73333333333334</v>
       </c>
     </row>
     <row r="197">
@@ -10312,13 +10312,13 @@
         </is>
       </c>
       <c r="H197">
-        <v>0.3125</v>
+        <v>0.6666666666666657</v>
       </c>
       <c r="I197">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J197">
-        <v>11.3</v>
+        <v>11.4</v>
       </c>
       <c r="K197">
         <v>11.2</v>
@@ -10337,7 +10337,7 @@
         <v>2015</v>
       </c>
       <c r="O197">
-        <v>11.465</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="198">
@@ -10366,13 +10366,13 @@
         </is>
       </c>
       <c r="H198">
-        <v>0.4166666666666661</v>
+        <v>0</v>
       </c>
       <c r="I198">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J198">
-        <v>11.7</v>
+        <v>11.6</v>
       </c>
       <c r="K198">
         <v>11.6</v>
@@ -10391,7 +10391,7 @@
         <v>2015</v>
       </c>
       <c r="O198">
-        <v>11.79333333333333</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="199">
@@ -10420,10 +10420,10 @@
         </is>
       </c>
       <c r="H199">
-        <v>0.6264568764568761</v>
+        <v>0.5545454545454543</v>
       </c>
       <c r="I199">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J199">
         <v>7.800000000000001</v>
@@ -10445,7 +10445,7 @@
         <v>2015</v>
       </c>
       <c r="O199">
-        <v>8.128717948717949</v>
+        <v>8.240909090909096</v>
       </c>
     </row>
     <row r="200">
@@ -10474,10 +10474,10 @@
         </is>
       </c>
       <c r="H200">
-        <v>1.770833333333332</v>
+        <v>1.583333333333331</v>
       </c>
       <c r="I200">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J200">
         <v>11.5</v>
@@ -10499,7 +10499,7 @@
         <v>2015</v>
       </c>
       <c r="O200">
-        <v>11.315</v>
+        <v>11.325</v>
       </c>
     </row>
     <row r="201">
@@ -10528,10 +10528,10 @@
         </is>
       </c>
       <c r="H201">
-        <v>-0.5357142857142865</v>
+        <v>-0.4999999999999993</v>
       </c>
       <c r="I201">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J201">
         <v>9.600000000000001</v>
@@ -10553,7 +10553,7 @@
         <v>2015</v>
       </c>
       <c r="O201">
-        <v>10.39428571428572</v>
+        <v>10.43333333333334</v>
       </c>
     </row>
     <row r="202">
@@ -10582,10 +10582,10 @@
         </is>
       </c>
       <c r="H202">
-        <v>2.194940476190477</v>
+        <v>2.004761904761905</v>
       </c>
       <c r="I202">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="J202">
         <v>10.4</v>
@@ -10607,7 +10607,7 @@
         <v>2015</v>
       </c>
       <c r="O202">
-        <v>9.797500000000005</v>
+        <v>9.857142857142856</v>
       </c>
     </row>
   </sheetData>

</xml_diff>